<commit_message>
update vercel.json fix xlsx download issue
</commit_message>
<xml_diff>
--- a/myswcautosar.xlsx
+++ b/myswcautosar.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\11_web\SWC_Maker\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andyzong\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAFD1E0E-21CB-4848-A727-E69D55F70253}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D86401F-685D-48EE-A52B-AC41C78A87E0}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12650" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="27">
   <si>
     <t>Direction</t>
   </si>
@@ -115,6 +115,22 @@
   </si>
   <si>
     <t>DoorMethod</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ReLeDoorSts3</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ReLeDoorSts4</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>SetSeatCmd</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>SeatMethod</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -588,7 +604,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{855DDDED-1E82-44DA-B35F-698B1AA9F0FA}">
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.4140625" customWidth="1"/>
@@ -756,13 +772,13 @@
         <v>1</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="G7" s="6" t="s">
         <v>11</v>
@@ -772,26 +788,73 @@
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A8" s="9"/>
-      <c r="B8" s="10" t="s">
+      <c r="A8" s="8"/>
+      <c r="B8" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="C8" s="10" t="s">
+      <c r="C8" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="H8" s="7" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9" s="9"/>
+      <c r="B9" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="C9" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="D8" s="10" t="s">
+      <c r="D9" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="E8" s="10" t="s">
+      <c r="E9" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="F8" s="10" t="s">
+      <c r="F9" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="G8" s="10" t="s">
+      <c r="G9" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="H8" s="11" t="s">
+      <c r="H9" s="11" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="B10" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="C10" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="D10" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="E10" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="F10" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="G10" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="H10" s="11" t="s">
         <v>12</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: support multiple elements per ClientServer interface and add float32 data type
  - ClientServer接口支持多个element/operation，通过Excel不同行定义
  - 同一端口下多个operation自动分组，一次性创建带所有com_spec的端口
  - 每个operation独立生成对应的runnable和operation invoked event
  - interface_data结构改为elements列表，支持同接口多element存储
  - create_clientserver_port支持传入operation列表（兼容单个字符串）
  - create_constants跳过ClientServer接口，仅为SenderReceiver创建初始值
  - 新增float32平台基础类型（IEEE754编码）和实现数据类型
</commit_message>
<xml_diff>
--- a/myswcautosar.xlsx
+++ b/myswcautosar.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andyzong\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\11_web\SWC_Maker\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D86401F-685D-48EE-A52B-AC41C78A87E0}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F34A603-9C60-40FE-AA82-FA8F8E36DFBF}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12650" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="31">
   <si>
     <t>Direction</t>
   </si>
@@ -131,6 +131,22 @@
   </si>
   <si>
     <t>SeatMethod</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>SetWindowCmd</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>CSwindowCmd</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>method1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>method2</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -169,7 +185,7 @@
       <charset val="134"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -179,6 +195,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -207,10 +235,74 @@
       <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin">
         <color indexed="64"/>
       </left>
-      <right/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
       <top style="thin">
         <color indexed="64"/>
       </top>
@@ -223,64 +315,6 @@
       <top style="thin">
         <color indexed="64"/>
       </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
@@ -290,39 +324,53 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -339,6 +387,280 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>31749</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>111125</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>450849</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>15875</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="Callout: Bent Line 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{161D001D-62F3-46D4-BF69-36658339215B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="12938124" y="587375"/>
+          <a:ext cx="2390775" cy="628650"/>
+        </a:xfrm>
+        <a:prstGeom prst="borderCallout2">
+          <a:avLst>
+            <a:gd name="adj1" fmla="val 18750"/>
+            <a:gd name="adj2" fmla="val -8333"/>
+            <a:gd name="adj3" fmla="val 18750"/>
+            <a:gd name="adj4" fmla="val -16667"/>
+            <a:gd name="adj5" fmla="val 68561"/>
+            <a:gd name="adj6" fmla="val -75294"/>
+          </a:avLst>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent4">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent4"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent4"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="zh-CN" altLang="en-US" sz="1100">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>生成普通</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" altLang="zh-CN" sz="1100">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>SR-Port</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="zh-CN" altLang="en-US" sz="1100">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>，</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" altLang="zh-CN" sz="1100">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>eg</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="zh-CN" altLang="en-US" sz="1100">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>：</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" altLang="zh-CN" sz="1100">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>rte_write_</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" altLang="zh-CN" sz="1100" b="0" i="0" u="none" strike="noStrike">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>LockCmd</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" altLang="zh-CN">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t> _LockCmd()</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="en-US" altLang="zh-CN" sz="1100">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>rte_read_VehSpd_VehSpd()</a:t>
+          </a:r>
+          <a:endParaRPr lang="zh-CN" altLang="en-US" sz="1100">
+            <a:solidFill>
+              <a:sysClr val="windowText" lastClr="000000"/>
+            </a:solidFill>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>31749</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>92075</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>349250</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="3" name="Callout: Bent Line 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{464977B5-BE93-4EF0-B38E-6E813EC8E7C5}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="12938124" y="1473200"/>
+          <a:ext cx="4260851" cy="631825"/>
+        </a:xfrm>
+        <a:prstGeom prst="borderCallout2">
+          <a:avLst>
+            <a:gd name="adj1" fmla="val 18750"/>
+            <a:gd name="adj2" fmla="val -8333"/>
+            <a:gd name="adj3" fmla="val 18750"/>
+            <a:gd name="adj4" fmla="val -16667"/>
+            <a:gd name="adj5" fmla="val 65546"/>
+            <a:gd name="adj6" fmla="val -37291"/>
+          </a:avLst>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent4">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent4"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent4"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="zh-CN" altLang="en-US" sz="1100">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>生成普通</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" altLang="zh-CN" sz="1100">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>server-runnable</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="zh-CN" altLang="en-US" sz="1100">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>，</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" altLang="zh-CN" sz="1100">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>eg</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="zh-CN" altLang="en-US" sz="1100">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>：</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" altLang="zh-CN" sz="1100">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>PSDContrl_SetSeatCmd_SeatMethod(uint8 invalue, uint8 outvalue)</a:t>
+          </a:r>
+          <a:endParaRPr lang="zh-CN" altLang="en-US" sz="1100">
+            <a:solidFill>
+              <a:sysClr val="windowText" lastClr="000000"/>
+            </a:solidFill>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -604,7 +926,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{855DDDED-1E82-44DA-B35F-698B1AA9F0FA}">
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.4140625" customWidth="1"/>
@@ -618,13 +940,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="12" t="s">
         <v>21</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="C1" s="3" t="s">
         <v>0</v>
       </c>
       <c r="D1" s="1" t="s">
@@ -645,30 +967,30 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="2"/>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G2" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="H2" s="5" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="5"/>
+      <c r="A3" s="2"/>
       <c r="B3" s="6" t="s">
         <v>2</v>
       </c>
@@ -692,7 +1014,7 @@
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" s="5"/>
+      <c r="A4" s="2"/>
       <c r="B4" s="6" t="s">
         <v>2</v>
       </c>
@@ -716,7 +1038,7 @@
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" s="5"/>
+      <c r="A5" s="2"/>
       <c r="B5" s="6" t="s">
         <v>2</v>
       </c>
@@ -740,7 +1062,7 @@
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A6" s="8"/>
+      <c r="A6" s="13"/>
       <c r="B6" s="6" t="s">
         <v>2</v>
       </c>
@@ -764,7 +1086,7 @@
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A7" s="8"/>
+      <c r="A7" s="13"/>
       <c r="B7" s="6" t="s">
         <v>2</v>
       </c>
@@ -788,31 +1110,31 @@
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A8" s="8"/>
-      <c r="B8" s="6" t="s">
+      <c r="A8" s="13"/>
+      <c r="B8" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C8" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="D8" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="E8" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="F8" s="6" t="s">
+      <c r="F8" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="G8" s="6" t="s">
+      <c r="G8" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="H8" s="7" t="s">
+      <c r="H8" s="9" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A9" s="9"/>
+      <c r="A9" s="13"/>
       <c r="B9" s="10" t="s">
         <v>2</v>
       </c>
@@ -836,6 +1158,7 @@
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A10" s="13"/>
       <c r="B10" s="10" t="s">
         <v>2</v>
       </c>
@@ -855,6 +1178,54 @@
         <v>18</v>
       </c>
       <c r="H10" s="11" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A11" s="13"/>
+      <c r="B11" s="14" t="s">
+        <v>2</v>
+      </c>
+      <c r="C11" s="14" t="s">
+        <v>9</v>
+      </c>
+      <c r="D11" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="E11" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="F11" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="G11" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="H11" s="16" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A12" s="13"/>
+      <c r="B12" s="14" t="s">
+        <v>2</v>
+      </c>
+      <c r="C12" s="14" t="s">
+        <v>9</v>
+      </c>
+      <c r="D12" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="E12" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="F12" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="G12" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="H12" s="16" t="s">
         <v>12</v>
       </c>
     </row>
@@ -862,5 +1233,6 @@
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
update workspace.write_documents(schema_version=46)，生成的 arxml 头部就会变成 AUTOSAR_00046.xsd
</commit_message>
<xml_diff>
--- a/myswcautosar.xlsx
+++ b/myswcautosar.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\11_web\SWC_Maker\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F34A603-9C60-40FE-AA82-FA8F8E36DFBF}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13D83312-A07C-48B4-9759-C4B8F2B452B3}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12650" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="28">
   <si>
     <t>Direction</t>
   </si>
@@ -90,10 +90,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>VehSpdVld</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>SetDoorCmd</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -115,14 +111,6 @@
   </si>
   <si>
     <t>DoorMethod</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>ReLeDoorSts3</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>ReLeDoorSts4</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -394,22 +382,22 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>10</xdr:col>
-      <xdr:colOff>31749</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>111125</xdr:rowOff>
+      <xdr:colOff>492125</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>92075</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>450849</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>15875</xdr:rowOff>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>234950</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="2" name="Callout: Bent Line 1">
+        <xdr:cNvPr id="5" name="Speech Bubble: Rectangle 4">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{161D001D-62F3-46D4-BF69-36658339215B}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{45B8773B-DF21-4A88-9748-B6E88E5004DA}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -417,93 +405,127 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="12938124" y="587375"/>
-          <a:ext cx="2390775" cy="628650"/>
+          <a:off x="13398500" y="1111250"/>
+          <a:ext cx="2371725" cy="631825"/>
         </a:xfrm>
-        <a:prstGeom prst="borderCallout2">
+        <a:prstGeom prst="wedgeRectCallout">
           <a:avLst>
-            <a:gd name="adj1" fmla="val 18750"/>
-            <a:gd name="adj2" fmla="val -8333"/>
-            <a:gd name="adj3" fmla="val 18750"/>
-            <a:gd name="adj4" fmla="val -16667"/>
-            <a:gd name="adj5" fmla="val 68561"/>
-            <a:gd name="adj6" fmla="val -75294"/>
+            <a:gd name="adj1" fmla="val -135576"/>
+            <a:gd name="adj2" fmla="val -77472"/>
           </a:avLst>
         </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent4">
+            <a:lumMod val="60000"/>
+            <a:lumOff val="40000"/>
+          </a:schemeClr>
+        </a:solidFill>
       </xdr:spPr>
       <xdr:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent4">
-            <a:shade val="50000"/>
-          </a:schemeClr>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent4"/>
         </a:lnRef>
-        <a:fillRef idx="1">
+        <a:fillRef idx="2">
           <a:schemeClr val="accent4"/>
         </a:fillRef>
-        <a:effectRef idx="0">
+        <a:effectRef idx="1">
           <a:schemeClr val="accent4"/>
         </a:effectRef>
         <a:fontRef idx="minor">
-          <a:schemeClr val="lt1"/>
+          <a:schemeClr val="dk1"/>
         </a:fontRef>
       </xdr:style>
       <xdr:txBody>
         <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
         <a:lstStyle/>
         <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="zh-CN" altLang="en-US" sz="1100">
-              <a:solidFill>
-                <a:sysClr val="windowText" lastClr="000000"/>
-              </a:solidFill>
+          <a:r>
+            <a:rPr lang="zh-CN" altLang="zh-CN" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
             </a:rPr>
             <a:t>生成普通</a:t>
           </a:r>
           <a:r>
             <a:rPr lang="en-US" altLang="zh-CN" sz="1100">
               <a:solidFill>
-                <a:sysClr val="windowText" lastClr="000000"/>
-              </a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
             </a:rPr>
             <a:t>SR-Port</a:t>
           </a:r>
           <a:r>
-            <a:rPr lang="zh-CN" altLang="en-US" sz="1100">
-              <a:solidFill>
-                <a:sysClr val="windowText" lastClr="000000"/>
-              </a:solidFill>
+            <a:rPr lang="zh-CN" altLang="zh-CN" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
             </a:rPr>
             <a:t>，</a:t>
           </a:r>
           <a:r>
             <a:rPr lang="en-US" altLang="zh-CN" sz="1100">
               <a:solidFill>
-                <a:sysClr val="windowText" lastClr="000000"/>
-              </a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
             </a:rPr>
             <a:t>eg</a:t>
           </a:r>
           <a:r>
-            <a:rPr lang="zh-CN" altLang="en-US" sz="1100">
-              <a:solidFill>
-                <a:sysClr val="windowText" lastClr="000000"/>
-              </a:solidFill>
+            <a:rPr lang="zh-CN" altLang="zh-CN" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
             </a:rPr>
             <a:t>：</a:t>
           </a:r>
-          <a:r>
-            <a:rPr lang="en-US" altLang="zh-CN" sz="1100">
-              <a:solidFill>
-                <a:sysClr val="windowText" lastClr="000000"/>
-              </a:solidFill>
+          <a:br>
+            <a:rPr lang="en-US" altLang="zh-CN" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+          </a:br>
+          <a:r>
+            <a:rPr lang="en-US" altLang="zh-CN" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
             </a:rPr>
             <a:t>rte_write_</a:t>
           </a:r>
           <a:r>
-            <a:rPr lang="en-US" altLang="zh-CN" sz="1100" b="0" i="0" u="none" strike="noStrike">
-              <a:solidFill>
-                <a:sysClr val="windowText" lastClr="000000"/>
+            <a:rPr lang="en-US" altLang="zh-CN" sz="1100" b="0" i="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
               </a:solidFill>
               <a:effectLst/>
               <a:latin typeface="+mn-lt"/>
@@ -513,29 +535,41 @@
             <a:t>LockCmd</a:t>
           </a:r>
           <a:r>
-            <a:rPr lang="en-US" altLang="zh-CN">
-              <a:solidFill>
-                <a:sysClr val="windowText" lastClr="000000"/>
-              </a:solidFill>
+            <a:rPr lang="en-US" altLang="zh-CN" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
             </a:rPr>
             <a:t> _LockCmd()</a:t>
           </a:r>
+          <a:endParaRPr lang="zh-CN" altLang="zh-CN">
+            <a:effectLst/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" altLang="zh-CN" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>rte_read_VehSpd_VehSpd()</a:t>
+          </a:r>
+          <a:endParaRPr lang="zh-CN" altLang="zh-CN">
+            <a:effectLst/>
+          </a:endParaRPr>
         </a:p>
         <a:p>
           <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" altLang="zh-CN" sz="1100">
-              <a:solidFill>
-                <a:sysClr val="windowText" lastClr="000000"/>
-              </a:solidFill>
-            </a:rPr>
-            <a:t>rte_read_VehSpd_VehSpd()</a:t>
-          </a:r>
-          <a:endParaRPr lang="zh-CN" altLang="en-US" sz="1100">
-            <a:solidFill>
-              <a:sysClr val="windowText" lastClr="000000"/>
-            </a:solidFill>
-          </a:endParaRPr>
+          <a:endParaRPr lang="zh-CN" altLang="en-US" sz="1100"/>
         </a:p>
       </xdr:txBody>
     </xdr:sp>
@@ -544,22 +578,22 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>10</xdr:col>
-      <xdr:colOff>31749</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>92075</xdr:rowOff>
+      <xdr:colOff>511175</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>63500</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>349250</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>254000</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="3" name="Callout: Bent Line 2">
+        <xdr:cNvPr id="6" name="Speech Bubble: Rectangle 5">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{464977B5-BE93-4EF0-B38E-6E813EC8E7C5}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8AEA1CCD-3930-4627-8430-8BF5B4BA07B6}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -567,94 +601,559 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="12938124" y="1473200"/>
-          <a:ext cx="4260851" cy="631825"/>
+          <a:off x="13417550" y="1806575"/>
+          <a:ext cx="2371725" cy="631825"/>
         </a:xfrm>
-        <a:prstGeom prst="borderCallout2">
+        <a:prstGeom prst="wedgeRectCallout">
           <a:avLst>
-            <a:gd name="adj1" fmla="val 18750"/>
-            <a:gd name="adj2" fmla="val -8333"/>
-            <a:gd name="adj3" fmla="val 18750"/>
-            <a:gd name="adj4" fmla="val -16667"/>
-            <a:gd name="adj5" fmla="val 65546"/>
-            <a:gd name="adj6" fmla="val -37291"/>
+            <a:gd name="adj1" fmla="val -141192"/>
+            <a:gd name="adj2" fmla="val -96104"/>
           </a:avLst>
         </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent4">
+            <a:lumMod val="60000"/>
+            <a:lumOff val="40000"/>
+          </a:schemeClr>
+        </a:solidFill>
       </xdr:spPr>
       <xdr:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent4">
-            <a:shade val="50000"/>
-          </a:schemeClr>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent4"/>
         </a:lnRef>
-        <a:fillRef idx="1">
+        <a:fillRef idx="2">
           <a:schemeClr val="accent4"/>
         </a:fillRef>
-        <a:effectRef idx="0">
+        <a:effectRef idx="1">
           <a:schemeClr val="accent4"/>
         </a:effectRef>
         <a:fontRef idx="minor">
-          <a:schemeClr val="lt1"/>
+          <a:schemeClr val="dk1"/>
         </a:fontRef>
       </xdr:style>
       <xdr:txBody>
         <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
         <a:lstStyle/>
         <a:p>
+          <a:r>
+            <a:rPr lang="zh-CN" altLang="zh-CN" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>生成普通</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" altLang="zh-CN" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>server-runnable</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="zh-CN" altLang="zh-CN" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>，</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" altLang="zh-CN" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>eg</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="zh-CN" altLang="zh-CN" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>：</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" altLang="zh-CN" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>PSDContrl_SetSeatCmd_SeatMethod(uint8 invalue, uint8 outvalue)</a:t>
+          </a:r>
+          <a:endParaRPr lang="zh-CN" altLang="zh-CN">
+            <a:effectLst/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
           <a:pPr algn="l"/>
+          <a:endParaRPr lang="zh-CN" altLang="en-US" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>126999</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>285750</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>38101</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="7" name="Speech Bubble: Rectangle 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{123B5392-F4A5-4D6C-A955-1DC6848013A0}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8480424" y="3086100"/>
+          <a:ext cx="4054476" cy="866776"/>
+        </a:xfrm>
+        <a:prstGeom prst="wedgeRectCallout">
+          <a:avLst>
+            <a:gd name="adj1" fmla="val -68312"/>
+            <a:gd name="adj2" fmla="val -167035"/>
+          </a:avLst>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent4">
+            <a:lumMod val="60000"/>
+            <a:lumOff val="40000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent4"/>
+        </a:lnRef>
+        <a:fillRef idx="2">
+          <a:schemeClr val="accent4"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent4"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="zh-CN" altLang="zh-CN" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>生成普通</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" altLang="zh-CN" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>server-runnable</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="zh-CN" altLang="zh-CN" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>，多个</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" altLang="zh-CN" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>method</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="zh-CN" altLang="zh-CN" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>在一个</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" altLang="zh-CN" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>CS</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="zh-CN" altLang="zh-CN" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>接口中，</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" altLang="zh-CN" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>eg</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="zh-CN" altLang="zh-CN" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>：</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" altLang="zh-CN" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>PSDContrl_CSwindowCmd_method1(uint8 invalue, uint8 outvalue)</a:t>
+          </a:r>
+          <a:endParaRPr lang="zh-CN" altLang="zh-CN">
+            <a:effectLst/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" altLang="zh-CN" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>PSDContrl_CSwindowCmd_method2(uint8 invalue, uint8 outvalue)</a:t>
+          </a:r>
+          <a:endParaRPr lang="zh-CN" altLang="zh-CN">
+            <a:effectLst/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" lvl="0" indent="0" algn="l" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+            <a:buClrTx/>
+            <a:buSzTx/>
+            <a:buFontTx/>
+            <a:buNone/>
+            <a:tabLst/>
+            <a:defRPr/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="en-US" altLang="zh-CN" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>PSDContrl_CSwindowCmd_method3(uint8 invalue, uint8 outvalue)</a:t>
+          </a:r>
+          <a:endParaRPr lang="zh-CN" altLang="zh-CN">
+            <a:effectLst/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="zh-CN" altLang="en-US" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>520700</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>225425</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>101600</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>15875</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="8" name="Speech Bubble: Rectangle 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3EAFBE9C-E3B2-4074-BF23-35877C222C20}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="13427075" y="225425"/>
+          <a:ext cx="2867025" cy="628650"/>
+        </a:xfrm>
+        <a:prstGeom prst="wedgeRectCallout">
+          <a:avLst>
+            <a:gd name="adj1" fmla="val -122632"/>
+            <a:gd name="adj2" fmla="val -47732"/>
+          </a:avLst>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent4">
+            <a:lumMod val="60000"/>
+            <a:lumOff val="40000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent4"/>
+        </a:lnRef>
+        <a:fillRef idx="2">
+          <a:schemeClr val="accent4"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent4"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
           <a:r>
             <a:rPr lang="zh-CN" altLang="en-US" sz="1100">
               <a:solidFill>
-                <a:sysClr val="windowText" lastClr="000000"/>
-              </a:solidFill>
-            </a:rPr>
-            <a:t>生成普通</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" altLang="zh-CN" sz="1100">
-              <a:solidFill>
-                <a:sysClr val="windowText" lastClr="000000"/>
-              </a:solidFill>
-            </a:rPr>
-            <a:t>server-runnable</a:t>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>仅支持</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="en-US" altLang="zh-CN" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+          </a:br>
+          <a:r>
+            <a:rPr lang="en-US" altLang="zh-CN" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>uint8</a:t>
           </a:r>
           <a:r>
             <a:rPr lang="zh-CN" altLang="en-US" sz="1100">
               <a:solidFill>
-                <a:sysClr val="windowText" lastClr="000000"/>
-              </a:solidFill>
-            </a:rPr>
-            <a:t>，</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" altLang="zh-CN" sz="1100">
-              <a:solidFill>
-                <a:sysClr val="windowText" lastClr="000000"/>
-              </a:solidFill>
-            </a:rPr>
-            <a:t>eg</a:t>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>、</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" altLang="zh-CN" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>uint16</a:t>
           </a:r>
           <a:r>
             <a:rPr lang="zh-CN" altLang="en-US" sz="1100">
               <a:solidFill>
-                <a:sysClr val="windowText" lastClr="000000"/>
-              </a:solidFill>
-            </a:rPr>
-            <a:t>：</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" altLang="zh-CN" sz="1100">
-              <a:solidFill>
-                <a:sysClr val="windowText" lastClr="000000"/>
-              </a:solidFill>
-            </a:rPr>
-            <a:t>PSDContrl_SetSeatCmd_SeatMethod(uint8 invalue, uint8 outvalue)</a:t>
-          </a:r>
-          <a:endParaRPr lang="zh-CN" altLang="en-US" sz="1100">
-            <a:solidFill>
-              <a:sysClr val="windowText" lastClr="000000"/>
-            </a:solidFill>
-          </a:endParaRPr>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>、</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" altLang="zh-CN" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>uint32</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="zh-CN" altLang="en-US" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>、</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" altLang="zh-CN" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>float32</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="zh-CN" altLang="en-US" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>、</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" altLang="zh-CN" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>boolean</a:t>
+          </a:r>
+          <a:endParaRPr lang="zh-CN" altLang="en-US" sz="1100"/>
         </a:p>
       </xdr:txBody>
     </xdr:sp>
@@ -926,7 +1425,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{855DDDED-1E82-44DA-B35F-698B1AA9F0FA}">
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.4140625" customWidth="1"/>
@@ -941,7 +1440,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>7</v>
@@ -1038,7 +1537,7 @@
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" s="2"/>
+      <c r="A5" s="13"/>
       <c r="B5" s="6" t="s">
         <v>2</v>
       </c>
@@ -1046,13 +1545,13 @@
         <v>1</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G5" s="6" t="s">
         <v>11</v>
@@ -1063,126 +1562,125 @@
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="13"/>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D6" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="E6" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="F6" s="6" t="s">
+      <c r="F6" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="G6" s="6" t="s">
+      <c r="G6" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="H6" s="7" t="s">
+      <c r="H6" s="9" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="13"/>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="C7" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="E7" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="F7" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="G7" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="H7" s="7" t="s">
+      <c r="C7" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="D7" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="E7" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="F7" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="G7" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="H7" s="11" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="13"/>
-      <c r="B8" s="8" t="s">
+      <c r="B8" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="C8" s="8" t="s">
-        <v>1</v>
-      </c>
-      <c r="D8" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="E8" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="F8" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="G8" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="H8" s="9" t="s">
+      <c r="C8" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="D8" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="E8" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="F8" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="G8" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="H8" s="11" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" s="13"/>
-      <c r="B9" s="10" t="s">
+      <c r="B9" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="C9" s="10" t="s">
+      <c r="C9" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="D9" s="10" t="s">
+      <c r="D9" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="E9" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="F9" s="15" t="s">
+        <v>26</v>
+      </c>
+      <c r="G9" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="E9" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="F9" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="G9" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="H9" s="11" t="s">
+      <c r="H9" s="16" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" s="13"/>
-      <c r="B10" s="10" t="s">
+      <c r="B10" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="C10" s="10" t="s">
+      <c r="C10" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="D10" s="10" t="s">
+      <c r="D10" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="E10" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="E10" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="F10" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="G10" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="H10" s="11" t="s">
+      <c r="F10" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="G10" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="H10" s="16" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A11" s="13"/>
       <c r="B11" s="14" t="s">
         <v>2</v>
       </c>
@@ -1190,43 +1688,19 @@
         <v>9</v>
       </c>
       <c r="D11" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="E11" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="F11" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="E11" s="15" t="s">
-        <v>28</v>
-      </c>
-      <c r="F11" s="15" t="s">
-        <v>29</v>
-      </c>
       <c r="G11" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="H11" s="16" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A12" s="13"/>
-      <c r="B12" s="14" t="s">
-        <v>2</v>
-      </c>
-      <c r="C12" s="14" t="s">
-        <v>9</v>
-      </c>
-      <c r="D12" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="E12" s="15" t="s">
-        <v>28</v>
-      </c>
-      <c r="F12" s="15" t="s">
-        <v>30</v>
-      </c>
-      <c r="G12" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="H12" s="16" t="s">
-        <v>12</v>
+        <v>17</v>
+      </c>
+      <c r="H11" s="14" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
● feat: add AUTOSAR struct (STRUCTURE) data type support
  Add a new optional "Struct" sheet in Excel template for defining
  composite data types. Struct members can reference primitive types
  or other structs (nested). Includes topological sort for dependency
  resolution, circular dependency detection, and RecordValueSpecification
  init values. Fully backward compatible - existing Excel files without
  Struct sheet work as before.
</commit_message>
<xml_diff>
--- a/myswcautosar.xlsx
+++ b/myswcautosar.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\11_web\SWC_Maker\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13D83312-A07C-48B4-9759-C4B8F2B452B3}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4A96521-1E5B-4503-92E1-C82D33924B15}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12650" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
+    <sheet name="Arch" sheetId="2" r:id="rId1"/>
+    <sheet name="Struct" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="45">
   <si>
     <t>Direction</t>
   </si>
@@ -136,13 +137,67 @@
   <si>
     <t>method2</t>
     <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>DoorStatus_T</t>
+  </si>
+  <si>
+    <t>DoorSts</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>DoorStsIf</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>DoorStatus_T</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>StructName</t>
+  </si>
+  <si>
+    <t>MemberName</t>
+  </si>
+  <si>
+    <t>MemberType</t>
+  </si>
+  <si>
+    <t>Position</t>
+  </si>
+  <si>
+    <t>uint8</t>
+  </si>
+  <si>
+    <t>LockSts</t>
+  </si>
+  <si>
+    <t>boolean</t>
+  </si>
+  <si>
+    <t>Speed</t>
+  </si>
+  <si>
+    <t>uint16</t>
+  </si>
+  <si>
+    <t>VehicleInfo_T</t>
+  </si>
+  <si>
+    <t>VehSpd</t>
+  </si>
+  <si>
+    <t>float32</t>
+  </si>
+  <si>
+    <t>DoorInfo</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -172,8 +227,16 @@
       <family val="2"/>
       <charset val="134"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="等线"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -198,8 +261,26 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="10">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -272,19 +353,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color indexed="64"/>
       </left>
@@ -298,21 +366,41 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
       <right/>
       <top style="thin">
         <color indexed="64"/>
       </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
+      <bottom/>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -323,41 +411,61 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1152,6 +1260,144 @@
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
             <a:t>boolean</a:t>
+          </a:r>
+          <a:endParaRPr lang="zh-CN" altLang="en-US" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>88899</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>171450</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>196850</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>44450</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="9" name="Speech Bubble: Rectangle 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EFBE1649-074C-4515-B6B2-BBC74EA2420A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="12995274" y="3362325"/>
+          <a:ext cx="4051301" cy="415925"/>
+        </a:xfrm>
+        <a:prstGeom prst="wedgeRectCallout">
+          <a:avLst>
+            <a:gd name="adj1" fmla="val -106672"/>
+            <a:gd name="adj2" fmla="val -286297"/>
+          </a:avLst>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent4">
+            <a:lumMod val="60000"/>
+            <a:lumOff val="40000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent4"/>
+        </a:lnRef>
+        <a:fillRef idx="2">
+          <a:schemeClr val="accent4"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent4"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" altLang="zh-CN" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>port</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="zh-CN" altLang="en-US" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>接口类型为</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" altLang="zh-CN" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>struct</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="zh-CN" altLang="en-US" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>类型，须在</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" altLang="zh-CN" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Struct</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="zh-CN" altLang="en-US" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>表单中定义</a:t>
           </a:r>
           <a:endParaRPr lang="zh-CN" altLang="en-US" sz="1100"/>
         </a:p>
@@ -1425,7 +1671,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{855DDDED-1E82-44DA-B35F-698B1AA9F0FA}">
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.4140625" customWidth="1"/>
@@ -1439,7 +1685,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="4" t="s">
         <v>20</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -1466,241 +1712,264 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="2"/>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="G2" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="H2" s="5" t="s">
+      <c r="H2" s="10" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="E3" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="F3" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="G3" s="6" t="s">
+      <c r="G3" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="H3" s="7" t="s">
+      <c r="H3" s="12" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="2"/>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="F4" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="G4" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="H4" s="7" t="s">
+      <c r="H4" s="12" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" s="13"/>
-      <c r="B5" s="6" t="s">
+      <c r="A5" s="5"/>
+      <c r="B5" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="E5" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="F5" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="G5" s="6" t="s">
+      <c r="G5" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="H5" s="7" t="s">
+      <c r="H5" s="12" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A6" s="13"/>
-      <c r="B6" s="8" t="s">
+      <c r="A6" s="5"/>
+      <c r="B6" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="8" t="s">
+      <c r="C6" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="D6" s="8" t="s">
+      <c r="D6" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="E6" s="8" t="s">
+      <c r="E6" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="F6" s="8" t="s">
+      <c r="F6" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="G6" s="8" t="s">
+      <c r="G6" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="H6" s="9" t="s">
+      <c r="H6" s="12" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A7" s="13"/>
-      <c r="B7" s="10" t="s">
+      <c r="A7" s="5"/>
+      <c r="B7" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="C7" s="10" t="s">
+      <c r="C7" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="D7" s="10" t="s">
+      <c r="D7" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="E7" s="10" t="s">
+      <c r="E7" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="F7" s="10" t="s">
+      <c r="F7" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="G7" s="10" t="s">
+      <c r="G7" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="H7" s="11" t="s">
+      <c r="H7" s="15" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A8" s="13"/>
-      <c r="B8" s="10" t="s">
+      <c r="A8" s="5"/>
+      <c r="B8" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="C8" s="10" t="s">
+      <c r="C8" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="D8" s="10" t="s">
+      <c r="D8" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="E8" s="10" t="s">
+      <c r="E8" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="F8" s="10" t="s">
+      <c r="F8" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="G8" s="10" t="s">
+      <c r="G8" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="H8" s="11" t="s">
+      <c r="H8" s="18" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A9" s="13"/>
-      <c r="B9" s="14" t="s">
+      <c r="A9" s="5"/>
+      <c r="B9" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="C9" s="14" t="s">
+      <c r="C9" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="D9" s="15" t="s">
+      <c r="D9" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="E9" s="15" t="s">
+      <c r="E9" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="F9" s="15" t="s">
+      <c r="F9" s="20" t="s">
         <v>26</v>
       </c>
-      <c r="G9" s="14" t="s">
+      <c r="G9" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="H9" s="16" t="s">
+      <c r="H9" s="21" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A10" s="13"/>
-      <c r="B10" s="14" t="s">
+      <c r="A10" s="5"/>
+      <c r="B10" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="C10" s="14" t="s">
+      <c r="C10" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="D10" s="15" t="s">
+      <c r="D10" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="E10" s="15" t="s">
+      <c r="E10" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="F10" s="15" t="s">
+      <c r="F10" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="G10" s="14" t="s">
+      <c r="G10" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="H10" s="16" t="s">
+      <c r="H10" s="21" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="B11" s="14" t="s">
+      <c r="B11" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="C11" s="14" t="s">
+      <c r="C11" s="23" t="s">
         <v>9</v>
       </c>
-      <c r="D11" s="15" t="s">
+      <c r="D11" s="23" t="s">
         <v>24</v>
       </c>
-      <c r="E11" s="15" t="s">
+      <c r="E11" s="23" t="s">
         <v>25</v>
       </c>
-      <c r="F11" s="15" t="s">
+      <c r="F11" s="23" t="s">
         <v>27</v>
       </c>
-      <c r="G11" s="14" t="s">
+      <c r="G11" s="23" t="s">
         <v>17</v>
       </c>
-      <c r="H11" s="14" t="s">
+      <c r="H11" s="24" t="s">
         <v>15</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="B12" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="C12" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D12" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="E12" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="F12" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="G12" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="H12" s="11" t="s">
+        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -1709,4 +1978,87 @@
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED218BF3-09CF-45B4-94C5-52D0387F6E36}">
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="19.9140625" customWidth="1"/>
+    <col min="2" max="2" width="18.83203125" customWidth="1"/>
+    <col min="3" max="3" width="21.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="39" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>28</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
add operation argument   - operation 参数名/方向/类型与 sheet 定义一致  - 支持 IN/OUT/INOUT 三种方向                                                       - 参数类型支持基本类型和结构体
</commit_message>
<xml_diff>
--- a/myswcautosar.xlsx
+++ b/myswcautosar.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\11_web\SWC_Maker\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4A96521-1E5B-4503-92E1-C82D33924B15}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57563837-95D3-4866-B3E3-34A3291BAF15}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12650" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12650" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Arch" sheetId="2" r:id="rId1"/>
+    <sheet name="Overview" sheetId="2" r:id="rId1"/>
     <sheet name="Struct" sheetId="3" r:id="rId2"/>
+    <sheet name="CSOperation" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="70">
   <si>
     <t>Direction</t>
   </si>
@@ -191,6 +192,84 @@
   </si>
   <si>
     <t>DoorInfo</t>
+  </si>
+  <si>
+    <t>InterfaceName</t>
+  </si>
+  <si>
+    <t>OperationName</t>
+  </si>
+  <si>
+    <t>ArgumentName</t>
+  </si>
+  <si>
+    <t>ArgumentDirection</t>
+  </si>
+  <si>
+    <t>ArgumentType</t>
+  </si>
+  <si>
+    <t>SetDoorCmd</t>
+  </si>
+  <si>
+    <t>DoorMethod</t>
+  </si>
+  <si>
+    <t>doorId</t>
+  </si>
+  <si>
+    <t>IN</t>
+  </si>
+  <si>
+    <t>doorCmd</t>
+  </si>
+  <si>
+    <t>result</t>
+  </si>
+  <si>
+    <t>OUT</t>
+  </si>
+  <si>
+    <t>SetSeatCmd</t>
+  </si>
+  <si>
+    <t>SeatMethod</t>
+  </si>
+  <si>
+    <t>seatPos</t>
+  </si>
+  <si>
+    <t>status</t>
+  </si>
+  <si>
+    <t>CSwindowCmd</t>
+  </si>
+  <si>
+    <t>method1</t>
+  </si>
+  <si>
+    <t>winId</t>
+  </si>
+  <si>
+    <t>method2</t>
+  </si>
+  <si>
+    <t>winPos</t>
+  </si>
+  <si>
+    <t>winCmd</t>
+  </si>
+  <si>
+    <t>na</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>NULL</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>float32</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -236,7 +315,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -279,8 +358,20 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="11">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -396,11 +487,48 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -441,15 +569,6 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -468,6 +587,51 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -688,13 +852,13 @@
       <xdr:col>10</xdr:col>
       <xdr:colOff>511175</xdr:colOff>
       <xdr:row>8</xdr:row>
-      <xdr:rowOff>63500</xdr:rowOff>
+      <xdr:rowOff>100292</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>14</xdr:col>
-      <xdr:colOff>254000</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>152400</xdr:rowOff>
+      <xdr:colOff>257175</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>6723</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -709,8 +873,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13417550" y="1806575"/>
-          <a:ext cx="2371725" cy="631825"/>
+          <a:off x="13409146" y="1837204"/>
+          <a:ext cx="2390588" cy="623607"/>
         </a:xfrm>
         <a:prstGeom prst="wedgeRectCallout">
           <a:avLst>
@@ -1671,7 +1835,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{855DDDED-1E82-44DA-B35F-698B1AA9F0FA}">
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:L36"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.4140625" customWidth="1"/>
@@ -1712,7 +1876,7 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="2"/>
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="33" t="s">
         <v>2</v>
       </c>
       <c r="C2" s="9" t="s">
@@ -1736,7 +1900,7 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
-      <c r="B3" s="11" t="s">
+      <c r="B3" s="34" t="s">
         <v>2</v>
       </c>
       <c r="C3" s="11" t="s">
@@ -1760,7 +1924,7 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="2"/>
-      <c r="B4" s="11" t="s">
+      <c r="B4" s="34" t="s">
         <v>2</v>
       </c>
       <c r="C4" s="11" t="s">
@@ -1779,12 +1943,12 @@
         <v>11</v>
       </c>
       <c r="H4" s="12" t="s">
-        <v>15</v>
+        <v>69</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="5"/>
-      <c r="B5" s="11" t="s">
+      <c r="B5" s="34" t="s">
         <v>2</v>
       </c>
       <c r="C5" s="11" t="s">
@@ -1803,30 +1967,30 @@
         <v>11</v>
       </c>
       <c r="H5" s="12" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="5"/>
-      <c r="B6" s="11" t="s">
+      <c r="B6" s="35" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="11" t="s">
+      <c r="C6" s="36" t="s">
         <v>1</v>
       </c>
-      <c r="D6" s="11" t="s">
+      <c r="D6" s="36" t="s">
         <v>19</v>
       </c>
-      <c r="E6" s="11" t="s">
+      <c r="E6" s="36" t="s">
         <v>19</v>
       </c>
-      <c r="F6" s="11" t="s">
+      <c r="F6" s="36" t="s">
         <v>19</v>
       </c>
-      <c r="G6" s="11" t="s">
+      <c r="G6" s="36" t="s">
         <v>11</v>
       </c>
-      <c r="H6" s="12" t="s">
+      <c r="H6" s="37" t="s">
         <v>12</v>
       </c>
     </row>
@@ -1851,125 +2015,130 @@
         <v>17</v>
       </c>
       <c r="H7" s="15" t="s">
-        <v>12</v>
+        <v>68</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="5"/>
-      <c r="B8" s="16" t="s">
+      <c r="B8" s="25" t="s">
         <v>2</v>
       </c>
-      <c r="C8" s="17" t="s">
+      <c r="C8" s="24" t="s">
         <v>9</v>
       </c>
-      <c r="D8" s="17" t="s">
+      <c r="D8" s="24" t="s">
         <v>22</v>
       </c>
-      <c r="E8" s="17" t="s">
+      <c r="E8" s="24" t="s">
         <v>22</v>
       </c>
-      <c r="F8" s="17" t="s">
+      <c r="F8" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="G8" s="17" t="s">
+      <c r="G8" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="H8" s="18" t="s">
-        <v>12</v>
+      <c r="H8" s="26" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" s="5"/>
-      <c r="B9" s="19" t="s">
+      <c r="B9" s="27" t="s">
         <v>2</v>
       </c>
-      <c r="C9" s="20" t="s">
+      <c r="C9" s="28" t="s">
         <v>9</v>
       </c>
-      <c r="D9" s="20" t="s">
+      <c r="D9" s="28" t="s">
         <v>24</v>
       </c>
-      <c r="E9" s="20" t="s">
+      <c r="E9" s="28" t="s">
         <v>25</v>
       </c>
-      <c r="F9" s="20" t="s">
+      <c r="F9" s="28" t="s">
         <v>26</v>
       </c>
-      <c r="G9" s="20" t="s">
+      <c r="G9" s="28" t="s">
         <v>17</v>
       </c>
-      <c r="H9" s="21" t="s">
-        <v>12</v>
+      <c r="H9" s="29" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" s="5"/>
-      <c r="B10" s="19" t="s">
+      <c r="B10" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="C10" s="20" t="s">
+      <c r="C10" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="D10" s="20" t="s">
+      <c r="D10" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="E10" s="20" t="s">
+      <c r="E10" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="F10" s="20" t="s">
+      <c r="F10" s="17" t="s">
         <v>27</v>
       </c>
-      <c r="G10" s="20" t="s">
+      <c r="G10" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="H10" s="21" t="s">
-        <v>12</v>
+      <c r="H10" s="18" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="B11" s="22" t="s">
+      <c r="B11" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="C11" s="23" t="s">
+      <c r="C11" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="D11" s="23" t="s">
+      <c r="D11" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="E11" s="23" t="s">
+      <c r="E11" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="F11" s="23" t="s">
+      <c r="F11" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="G11" s="23" t="s">
+      <c r="G11" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="H11" s="24" t="s">
-        <v>15</v>
+      <c r="H11" s="21" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="B12" s="11" t="s">
+      <c r="B12" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="C12" s="11" t="s">
+      <c r="C12" s="31" t="s">
         <v>1</v>
       </c>
-      <c r="D12" s="11" t="s">
+      <c r="D12" s="31" t="s">
         <v>29</v>
       </c>
-      <c r="E12" s="11" t="s">
+      <c r="E12" s="31" t="s">
         <v>30</v>
       </c>
-      <c r="F12" s="11" t="s">
+      <c r="F12" s="31" t="s">
         <v>29</v>
       </c>
-      <c r="G12" s="11" t="s">
+      <c r="G12" s="31" t="s">
         <v>11</v>
       </c>
-      <c r="H12" s="11" t="s">
+      <c r="H12" s="32" t="s">
         <v>31</v>
+      </c>
+    </row>
+    <row r="36" spans="12:12" x14ac:dyDescent="0.3">
+      <c r="L36" t="s">
+        <v>67</v>
       </c>
     </row>
   </sheetData>
@@ -2061,4 +2230,210 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8EBC7E7-ACF2-45B7-A880-C362C35F7623}">
+  <dimension ref="A1:E11"/>
+  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="22.9140625" customWidth="1"/>
+    <col min="2" max="2" width="18.25" customWidth="1"/>
+    <col min="3" max="3" width="15.75" customWidth="1"/>
+    <col min="4" max="4" width="16.6640625" customWidth="1"/>
+    <col min="5" max="5" width="19.58203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" s="38" t="s">
+        <v>50</v>
+      </c>
+      <c r="B2" s="38" t="s">
+        <v>51</v>
+      </c>
+      <c r="C2" s="38" t="s">
+        <v>52</v>
+      </c>
+      <c r="D2" s="38" t="s">
+        <v>53</v>
+      </c>
+      <c r="E2" s="38" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" s="38" t="s">
+        <v>50</v>
+      </c>
+      <c r="B3" s="38" t="s">
+        <v>51</v>
+      </c>
+      <c r="C3" s="38" t="s">
+        <v>54</v>
+      </c>
+      <c r="D3" s="38" t="s">
+        <v>53</v>
+      </c>
+      <c r="E3" s="38" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" s="38" t="s">
+        <v>50</v>
+      </c>
+      <c r="B4" s="38" t="s">
+        <v>51</v>
+      </c>
+      <c r="C4" s="38" t="s">
+        <v>55</v>
+      </c>
+      <c r="D4" s="38" t="s">
+        <v>56</v>
+      </c>
+      <c r="E4" s="38" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" s="22" t="s">
+        <v>57</v>
+      </c>
+      <c r="B5" s="22" t="s">
+        <v>58</v>
+      </c>
+      <c r="C5" s="22" t="s">
+        <v>59</v>
+      </c>
+      <c r="D5" s="22" t="s">
+        <v>53</v>
+      </c>
+      <c r="E5" s="22" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" s="22" t="s">
+        <v>57</v>
+      </c>
+      <c r="B6" s="22" t="s">
+        <v>58</v>
+      </c>
+      <c r="C6" s="22" t="s">
+        <v>60</v>
+      </c>
+      <c r="D6" s="22" t="s">
+        <v>56</v>
+      </c>
+      <c r="E6" s="22" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" s="23" t="s">
+        <v>61</v>
+      </c>
+      <c r="B7" s="23" t="s">
+        <v>62</v>
+      </c>
+      <c r="C7" s="23" t="s">
+        <v>63</v>
+      </c>
+      <c r="D7" s="23" t="s">
+        <v>53</v>
+      </c>
+      <c r="E7" s="23" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" s="23" t="s">
+        <v>61</v>
+      </c>
+      <c r="B8" s="23" t="s">
+        <v>62</v>
+      </c>
+      <c r="C8" s="23" t="s">
+        <v>55</v>
+      </c>
+      <c r="D8" s="23" t="s">
+        <v>56</v>
+      </c>
+      <c r="E8" s="23" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9" s="23" t="s">
+        <v>61</v>
+      </c>
+      <c r="B9" s="23" t="s">
+        <v>64</v>
+      </c>
+      <c r="C9" s="23" t="s">
+        <v>65</v>
+      </c>
+      <c r="D9" s="23" t="s">
+        <v>53</v>
+      </c>
+      <c r="E9" s="23" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10" s="23" t="s">
+        <v>61</v>
+      </c>
+      <c r="B10" s="23" t="s">
+        <v>64</v>
+      </c>
+      <c r="C10" s="23" t="s">
+        <v>66</v>
+      </c>
+      <c r="D10" s="23" t="s">
+        <v>53</v>
+      </c>
+      <c r="E10" s="23" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11" s="23" t="s">
+        <v>61</v>
+      </c>
+      <c r="B11" s="23" t="s">
+        <v>64</v>
+      </c>
+      <c r="C11" s="23" t="s">
+        <v>55</v>
+      </c>
+      <c r="D11" s="23" t="s">
+        <v>56</v>
+      </c>
+      <c r="E11" s="23" t="s">
+        <v>36</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
update PSDContrl to VehContrl
</commit_message>
<xml_diff>
--- a/myswcautosar.xlsx
+++ b/myswcautosar.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\11_web\SWC_Maker\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\00_web\SWC_Maker\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57563837-95D3-4866-B3E3-34A3291BAF15}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B22EC2F3-4CA3-4552-AFAE-302B628473BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12650" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2115" yWindow="930" windowWidth="24435" windowHeight="14025" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="2" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="71">
   <si>
     <t>Direction</t>
   </si>
@@ -36,10 +36,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>PSDContrl</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>InterfaceName</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -269,6 +265,13 @@
   </si>
   <si>
     <t>float32</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>VehContrl</t>
+  </si>
+  <si>
+    <t>VehContrl</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -276,7 +279,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -528,12 +531,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -542,7 +545,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -554,7 +556,7 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -572,7 +574,7 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -589,7 +591,7 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -634,7 +636,7 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="常规" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -855,8 +857,8 @@
       <xdr:rowOff>100292</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>14</xdr:col>
-      <xdr:colOff>257175</xdr:colOff>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>56029</xdr:colOff>
       <xdr:row>12</xdr:row>
       <xdr:rowOff>6723</xdr:rowOff>
     </xdr:to>
@@ -873,8 +875,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13409146" y="1837204"/>
-          <a:ext cx="2390588" cy="623607"/>
+          <a:off x="13453969" y="1837204"/>
+          <a:ext cx="4329766" cy="623607"/>
         </a:xfrm>
         <a:prstGeom prst="wedgeRectCallout">
           <a:avLst>
@@ -944,6 +946,18 @@
             <a:t>，</a:t>
           </a:r>
           <a:r>
+            <a:rPr lang="zh-CN" altLang="en-US" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>在</a:t>
+          </a:r>
+          <a:r>
             <a:rPr lang="en-US" altLang="zh-CN" sz="1100">
               <a:solidFill>
                 <a:schemeClr val="dk1"/>
@@ -953,6 +967,30 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
+            <a:t>CSOperation</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="zh-CN" altLang="en-US" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>表单定义形参，</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" altLang="zh-CN" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
             <a:t>eg</a:t>
           </a:r>
           <a:r>
@@ -977,7 +1015,31 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>PSDContrl_SetSeatCmd_SeatMethod(uint8 invalue, uint8 outvalue)</a:t>
+            <a:t>VehContrl_SetSeatCmd_SeatMethod(ArgumentType name,</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" altLang="zh-CN" sz="1100" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> ..., ...</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" altLang="zh-CN" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>)</a:t>
           </a:r>
           <a:endParaRPr lang="zh-CN" altLang="zh-CN">
             <a:effectLst/>
@@ -1169,7 +1231,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>PSDContrl_CSwindowCmd_method1(uint8 invalue, uint8 outvalue)</a:t>
+            <a:t>VehContrl_CSwindowCmd_method1(ArgumentType name, ..., ...)</a:t>
           </a:r>
           <a:endParaRPr lang="zh-CN" altLang="zh-CN">
             <a:effectLst/>
@@ -1186,30 +1248,13 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>PSDContrl_CSwindowCmd_method2(uint8 invalue, uint8 outvalue)</a:t>
+            <a:t>VehContrl_CSwindowCmd_method2(ArgumentType name, ..., ...)</a:t>
           </a:r>
           <a:endParaRPr lang="zh-CN" altLang="zh-CN">
             <a:effectLst/>
           </a:endParaRPr>
         </a:p>
         <a:p>
-          <a:pPr marL="0" marR="0" lvl="0" indent="0" algn="l" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
-            <a:lnSpc>
-              <a:spcPct val="100000"/>
-            </a:lnSpc>
-            <a:spcBef>
-              <a:spcPts val="0"/>
-            </a:spcBef>
-            <a:spcAft>
-              <a:spcPts val="0"/>
-            </a:spcAft>
-            <a:buClrTx/>
-            <a:buSzTx/>
-            <a:buFontTx/>
-            <a:buNone/>
-            <a:tabLst/>
-            <a:defRPr/>
-          </a:pPr>
           <a:r>
             <a:rPr lang="en-US" altLang="zh-CN" sz="1100">
               <a:solidFill>
@@ -1220,7 +1265,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>PSDContrl_CSwindowCmd_method3(uint8 invalue, uint8 outvalue)</a:t>
+            <a:t>VehContrl_CSwindowCmd_method3(ArgumentType name, ..., ...)</a:t>
           </a:r>
           <a:endParaRPr lang="zh-CN" altLang="zh-CN">
             <a:effectLst/>
@@ -1304,7 +1349,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>仅支持</a:t>
+            <a:t>支持</a:t>
           </a:r>
           <a:br>
             <a:rPr lang="en-US" altLang="zh-CN" sz="1100">
@@ -1327,103 +1372,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>uint8</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="zh-CN" altLang="en-US" sz="1100">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>、</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" altLang="zh-CN" sz="1100">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>uint16</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="zh-CN" altLang="en-US" sz="1100">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>、</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" altLang="zh-CN" sz="1100">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>uint32</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="zh-CN" altLang="en-US" sz="1100">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>、</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" altLang="zh-CN" sz="1100">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>float32</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="zh-CN" altLang="en-US" sz="1100">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>、</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" altLang="zh-CN" sz="1100">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>boolean</a:t>
+            <a:t>uint8,uint16,uint32,float32,boolean,Struct</a:t>
           </a:r>
           <a:endParaRPr lang="zh-CN" altLang="en-US" sz="1100"/>
         </a:p>
@@ -1836,309 +1785,303 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{855DDDED-1E82-44DA-B35F-698B1AA9F0FA}">
   <dimension ref="A1:L36"/>
-  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="14.4140625" customWidth="1"/>
-    <col min="2" max="2" width="13.1640625" customWidth="1"/>
-    <col min="3" max="3" width="14.6640625" customWidth="1"/>
-    <col min="4" max="4" width="20.6640625" customWidth="1"/>
-    <col min="5" max="5" width="28.9140625" customWidth="1"/>
+    <col min="1" max="1" width="14.375" customWidth="1"/>
+    <col min="2" max="2" width="13.125" customWidth="1"/>
+    <col min="3" max="3" width="14.625" customWidth="1"/>
+    <col min="4" max="4" width="20.625" customWidth="1"/>
+    <col min="5" max="5" width="28.875" customWidth="1"/>
     <col min="6" max="6" width="18" customWidth="1"/>
-    <col min="7" max="7" width="18.9140625" customWidth="1"/>
-    <col min="8" max="8" width="23.6640625" customWidth="1"/>
+    <col min="7" max="7" width="18.875" customWidth="1"/>
+    <col min="8" max="8" width="23.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="37.5" customHeight="1">
       <c r="A1" s="4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C1" s="3" t="s">
         <v>0</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="1" t="s">
-        <v>5</v>
-      </c>
       <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
+      <c r="A2" s="2"/>
+      <c r="B2" s="32" t="s">
+        <v>69</v>
+      </c>
+      <c r="C2" s="8" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="2"/>
-      <c r="B2" s="33" t="s">
-        <v>2</v>
-      </c>
-      <c r="C2" s="9" t="s">
+      <c r="D2" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="9" t="s">
+      <c r="E2" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="G2" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="9" t="s">
+      <c r="H2" s="9" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
+      <c r="A3" s="2"/>
+      <c r="B3" s="33" t="s">
+        <v>69</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="G3" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="F2" s="9" t="s">
+      <c r="H3" s="11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
+      <c r="A4" s="2"/>
+      <c r="B4" s="33" t="s">
+        <v>70</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="D4" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F4" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="G4" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="G2" s="9" t="s">
+      <c r="H4" s="11" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
+      <c r="B5" s="33" t="s">
+        <v>69</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="E5" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="F5" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="G5" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H5" s="11" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
+      <c r="B6" s="34" t="s">
+        <v>69</v>
+      </c>
+      <c r="C6" s="35" t="s">
+        <v>1</v>
+      </c>
+      <c r="D6" s="35" t="s">
+        <v>18</v>
+      </c>
+      <c r="E6" s="35" t="s">
+        <v>18</v>
+      </c>
+      <c r="F6" s="35" t="s">
+        <v>18</v>
+      </c>
+      <c r="G6" s="35" t="s">
+        <v>10</v>
+      </c>
+      <c r="H6" s="36" t="s">
         <v>11</v>
       </c>
-      <c r="H2" s="10" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="2"/>
-      <c r="B3" s="34" t="s">
-        <v>2</v>
-      </c>
-      <c r="C3" s="11" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="E3" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="F3" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="G3" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="H3" s="12" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" s="2"/>
-      <c r="B4" s="34" t="s">
-        <v>2</v>
-      </c>
-      <c r="C4" s="11" t="s">
+    </row>
+    <row r="7" spans="1:8">
+      <c r="B7" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="C7" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="D7" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="E7" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="F7" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="G7" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="H7" s="14" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
+      <c r="B8" s="24" t="s">
+        <v>69</v>
+      </c>
+      <c r="C8" s="23" t="s">
+        <v>8</v>
+      </c>
+      <c r="D8" s="23" t="s">
+        <v>21</v>
+      </c>
+      <c r="E8" s="23" t="s">
+        <v>21</v>
+      </c>
+      <c r="F8" s="23" t="s">
+        <v>22</v>
+      </c>
+      <c r="G8" s="23" t="s">
+        <v>16</v>
+      </c>
+      <c r="H8" s="25" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8">
+      <c r="B9" s="26" t="s">
+        <v>69</v>
+      </c>
+      <c r="C9" s="27" t="s">
+        <v>8</v>
+      </c>
+      <c r="D9" s="27" t="s">
+        <v>23</v>
+      </c>
+      <c r="E9" s="27" t="s">
+        <v>24</v>
+      </c>
+      <c r="F9" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="G9" s="27" t="s">
+        <v>16</v>
+      </c>
+      <c r="H9" s="28" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8">
+      <c r="B10" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="C10" s="16" t="s">
+        <v>8</v>
+      </c>
+      <c r="D10" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="E10" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="F10" s="16" t="s">
+        <v>26</v>
+      </c>
+      <c r="G10" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="H10" s="17" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8">
+      <c r="B11" s="18" t="s">
+        <v>69</v>
+      </c>
+      <c r="C11" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="D11" s="19" t="s">
+        <v>23</v>
+      </c>
+      <c r="E11" s="19" t="s">
+        <v>24</v>
+      </c>
+      <c r="F11" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="G11" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="H11" s="20" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8">
+      <c r="B12" s="29" t="s">
+        <v>69</v>
+      </c>
+      <c r="C12" s="30" t="s">
         <v>1</v>
       </c>
-      <c r="D4" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="E4" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="F4" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="G4" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="H4" s="12" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" s="5"/>
-      <c r="B5" s="34" t="s">
-        <v>2</v>
-      </c>
-      <c r="C5" s="11" t="s">
-        <v>1</v>
-      </c>
-      <c r="D5" s="11" t="s">
-        <v>18</v>
-      </c>
-      <c r="E5" s="11" t="s">
-        <v>18</v>
-      </c>
-      <c r="F5" s="11" t="s">
-        <v>18</v>
-      </c>
-      <c r="G5" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="H5" s="12" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A6" s="5"/>
-      <c r="B6" s="35" t="s">
-        <v>2</v>
-      </c>
-      <c r="C6" s="36" t="s">
-        <v>1</v>
-      </c>
-      <c r="D6" s="36" t="s">
-        <v>19</v>
-      </c>
-      <c r="E6" s="36" t="s">
-        <v>19</v>
-      </c>
-      <c r="F6" s="36" t="s">
-        <v>19</v>
-      </c>
-      <c r="G6" s="36" t="s">
-        <v>11</v>
-      </c>
-      <c r="H6" s="37" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A7" s="5"/>
-      <c r="B7" s="13" t="s">
-        <v>2</v>
-      </c>
-      <c r="C7" s="14" t="s">
-        <v>9</v>
-      </c>
-      <c r="D7" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="E7" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="F7" s="14" t="s">
-        <v>21</v>
-      </c>
-      <c r="G7" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="H7" s="15" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A8" s="5"/>
-      <c r="B8" s="25" t="s">
-        <v>2</v>
-      </c>
-      <c r="C8" s="24" t="s">
-        <v>9</v>
-      </c>
-      <c r="D8" s="24" t="s">
-        <v>22</v>
-      </c>
-      <c r="E8" s="24" t="s">
-        <v>22</v>
-      </c>
-      <c r="F8" s="24" t="s">
-        <v>23</v>
-      </c>
-      <c r="G8" s="24" t="s">
-        <v>17</v>
-      </c>
-      <c r="H8" s="26" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A9" s="5"/>
-      <c r="B9" s="27" t="s">
-        <v>2</v>
-      </c>
-      <c r="C9" s="28" t="s">
-        <v>9</v>
-      </c>
-      <c r="D9" s="28" t="s">
-        <v>24</v>
-      </c>
-      <c r="E9" s="28" t="s">
-        <v>25</v>
-      </c>
-      <c r="F9" s="28" t="s">
-        <v>26</v>
-      </c>
-      <c r="G9" s="28" t="s">
-        <v>17</v>
-      </c>
-      <c r="H9" s="29" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A10" s="5"/>
-      <c r="B10" s="16" t="s">
-        <v>2</v>
-      </c>
-      <c r="C10" s="17" t="s">
-        <v>9</v>
-      </c>
-      <c r="D10" s="17" t="s">
-        <v>24</v>
-      </c>
-      <c r="E10" s="17" t="s">
-        <v>25</v>
-      </c>
-      <c r="F10" s="17" t="s">
-        <v>27</v>
-      </c>
-      <c r="G10" s="17" t="s">
-        <v>17</v>
-      </c>
-      <c r="H10" s="18" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="B11" s="19" t="s">
-        <v>2</v>
-      </c>
-      <c r="C11" s="20" t="s">
-        <v>9</v>
-      </c>
-      <c r="D11" s="20" t="s">
-        <v>24</v>
-      </c>
-      <c r="E11" s="20" t="s">
-        <v>25</v>
-      </c>
-      <c r="F11" s="20" t="s">
-        <v>27</v>
-      </c>
-      <c r="G11" s="20" t="s">
-        <v>17</v>
-      </c>
-      <c r="H11" s="21" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="B12" s="30" t="s">
-        <v>2</v>
-      </c>
-      <c r="C12" s="31" t="s">
-        <v>1</v>
-      </c>
-      <c r="D12" s="31" t="s">
+      <c r="D12" s="30" t="s">
+        <v>28</v>
+      </c>
+      <c r="E12" s="30" t="s">
         <v>29</v>
       </c>
-      <c r="E12" s="31" t="s">
+      <c r="F12" s="30" t="s">
+        <v>28</v>
+      </c>
+      <c r="G12" s="30" t="s">
+        <v>10</v>
+      </c>
+      <c r="H12" s="31" t="s">
         <v>30</v>
       </c>
-      <c r="F12" s="31" t="s">
-        <v>29</v>
-      </c>
-      <c r="G12" s="31" t="s">
-        <v>11</v>
-      </c>
-      <c r="H12" s="32" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="36" spans="12:12" x14ac:dyDescent="0.3">
+    </row>
+    <row r="36" spans="12:12">
       <c r="L36" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>
@@ -2152,77 +2095,77 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED218BF3-09CF-45B4-94C5-52D0387F6E36}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="19.9140625" customWidth="1"/>
-    <col min="2" max="2" width="18.83203125" customWidth="1"/>
-    <col min="3" max="3" width="21.6640625" customWidth="1"/>
+    <col min="1" max="1" width="19.875" customWidth="1"/>
+    <col min="2" max="2" width="18.875" customWidth="1"/>
+    <col min="3" max="3" width="21.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="39" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="8" t="s">
+    <row r="1" spans="1:3" ht="39" customHeight="1">
+      <c r="A1" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="B1" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="C1" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="C1" s="8" t="s">
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" s="6" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="B2" s="7" t="s">
+      <c r="C2" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="C2" s="7" t="s">
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3" s="6" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="B3" s="7" t="s">
+      <c r="C3" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="C3" s="7" t="s">
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" s="6" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="B4" s="7" t="s">
+      <c r="C4" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="C4" s="7" t="s">
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" s="5" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="6" t="s">
+      <c r="B5" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="C5" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="C5" s="6" t="s">
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B6" s="5" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>28</v>
+      <c r="C6" s="5" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -2235,200 +2178,200 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8EBC7E7-ACF2-45B7-A880-C362C35F7623}">
   <dimension ref="A1:E11"/>
-  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="22.9140625" customWidth="1"/>
+    <col min="1" max="1" width="22.875" customWidth="1"/>
     <col min="2" max="2" width="18.25" customWidth="1"/>
     <col min="3" max="3" width="15.75" customWidth="1"/>
-    <col min="4" max="4" width="16.6640625" customWidth="1"/>
-    <col min="5" max="5" width="19.58203125" customWidth="1"/>
+    <col min="4" max="4" width="16.625" customWidth="1"/>
+    <col min="5" max="5" width="19.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="8" t="s">
+    <row r="1" spans="1:5" ht="45" customHeight="1">
+      <c r="A1" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="B1" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="C1" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="D1" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="E1" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="E1" s="8" t="s">
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" s="37" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A2" s="38" t="s">
+      <c r="B2" s="37" t="s">
         <v>50</v>
       </c>
-      <c r="B2" s="38" t="s">
+      <c r="C2" s="37" t="s">
         <v>51</v>
       </c>
-      <c r="C2" s="38" t="s">
+      <c r="D2" s="37" t="s">
         <v>52</v>
       </c>
-      <c r="D2" s="38" t="s">
+      <c r="E2" s="37" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" s="37" t="s">
+        <v>49</v>
+      </c>
+      <c r="B3" s="37" t="s">
+        <v>50</v>
+      </c>
+      <c r="C3" s="37" t="s">
         <v>53</v>
       </c>
-      <c r="E2" s="38" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3" s="38" t="s">
+      <c r="D3" s="37" t="s">
+        <v>52</v>
+      </c>
+      <c r="E3" s="37" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" s="37" t="s">
+        <v>49</v>
+      </c>
+      <c r="B4" s="37" t="s">
         <v>50</v>
       </c>
-      <c r="B3" s="38" t="s">
-        <v>51</v>
-      </c>
-      <c r="C3" s="38" t="s">
+      <c r="C4" s="37" t="s">
         <v>54</v>
       </c>
-      <c r="D3" s="38" t="s">
-        <v>53</v>
-      </c>
-      <c r="E3" s="38" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A4" s="38" t="s">
-        <v>50</v>
-      </c>
-      <c r="B4" s="38" t="s">
-        <v>51</v>
-      </c>
-      <c r="C4" s="38" t="s">
+      <c r="D4" s="37" t="s">
         <v>55</v>
       </c>
-      <c r="D4" s="38" t="s">
+      <c r="E4" s="37" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" s="21" t="s">
         <v>56</v>
       </c>
-      <c r="E4" s="38" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A5" s="22" t="s">
+      <c r="B5" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="B5" s="22" t="s">
+      <c r="C5" s="21" t="s">
         <v>58</v>
       </c>
-      <c r="C5" s="22" t="s">
+      <c r="D5" s="21" t="s">
+        <v>52</v>
+      </c>
+      <c r="E5" s="21" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" s="21" t="s">
+        <v>56</v>
+      </c>
+      <c r="B6" s="21" t="s">
+        <v>57</v>
+      </c>
+      <c r="C6" s="21" t="s">
         <v>59</v>
       </c>
-      <c r="D5" s="22" t="s">
-        <v>53</v>
-      </c>
-      <c r="E5" s="22" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A6" s="22" t="s">
-        <v>57</v>
-      </c>
-      <c r="B6" s="22" t="s">
-        <v>58</v>
-      </c>
-      <c r="C6" s="22" t="s">
+      <c r="D6" s="21" t="s">
+        <v>55</v>
+      </c>
+      <c r="E6" s="21" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7" s="22" t="s">
         <v>60</v>
       </c>
-      <c r="D6" s="22" t="s">
-        <v>56</v>
-      </c>
-      <c r="E6" s="22" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A7" s="23" t="s">
+      <c r="B7" s="22" t="s">
         <v>61</v>
       </c>
-      <c r="B7" s="23" t="s">
+      <c r="C7" s="22" t="s">
         <v>62</v>
       </c>
-      <c r="C7" s="23" t="s">
+      <c r="D7" s="22" t="s">
+        <v>52</v>
+      </c>
+      <c r="E7" s="22" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
+      <c r="A8" s="22" t="s">
+        <v>60</v>
+      </c>
+      <c r="B8" s="22" t="s">
+        <v>61</v>
+      </c>
+      <c r="C8" s="22" t="s">
+        <v>54</v>
+      </c>
+      <c r="D8" s="22" t="s">
+        <v>55</v>
+      </c>
+      <c r="E8" s="22" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
+      <c r="A9" s="22" t="s">
+        <v>60</v>
+      </c>
+      <c r="B9" s="22" t="s">
         <v>63</v>
       </c>
-      <c r="D7" s="23" t="s">
-        <v>53</v>
-      </c>
-      <c r="E7" s="23" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A8" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="B8" s="23" t="s">
-        <v>62</v>
-      </c>
-      <c r="C8" s="23" t="s">
+      <c r="C9" s="22" t="s">
+        <v>64</v>
+      </c>
+      <c r="D9" s="22" t="s">
+        <v>52</v>
+      </c>
+      <c r="E9" s="22" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="A10" s="22" t="s">
+        <v>60</v>
+      </c>
+      <c r="B10" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C10" s="22" t="s">
+        <v>65</v>
+      </c>
+      <c r="D10" s="22" t="s">
+        <v>52</v>
+      </c>
+      <c r="E10" s="22" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
+      <c r="A11" s="22" t="s">
+        <v>60</v>
+      </c>
+      <c r="B11" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C11" s="22" t="s">
+        <v>54</v>
+      </c>
+      <c r="D11" s="22" t="s">
         <v>55</v>
       </c>
-      <c r="D8" s="23" t="s">
-        <v>56</v>
-      </c>
-      <c r="E8" s="23" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A9" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="B9" s="23" t="s">
-        <v>64</v>
-      </c>
-      <c r="C9" s="23" t="s">
-        <v>65</v>
-      </c>
-      <c r="D9" s="23" t="s">
-        <v>53</v>
-      </c>
-      <c r="E9" s="23" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A10" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="B10" s="23" t="s">
-        <v>64</v>
-      </c>
-      <c r="C10" s="23" t="s">
-        <v>66</v>
-      </c>
-      <c r="D10" s="23" t="s">
-        <v>53</v>
-      </c>
-      <c r="E10" s="23" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A11" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="B11" s="23" t="s">
-        <v>64</v>
-      </c>
-      <c r="C11" s="23" t="s">
-        <v>55</v>
-      </c>
-      <c r="D11" s="23" t="s">
-        <v>56</v>
-      </c>
-      <c r="E11" s="23" t="s">
-        <v>36</v>
+      <c r="E11" s="22" t="s">
+        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>